<commit_message>
feat: add course textbook governance rules
</commit_message>
<xml_diff>
--- a/docs/ai-governance/20260605数据清单.xlsx
+++ b/docs/ai-governance/20260605数据清单.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="14605" activeTab="1"/>
+    <workbookView windowHeight="14605"/>
   </bookViews>
   <sheets>
     <sheet name="对应分类说明" sheetId="1" r:id="rId1"/>
@@ -114,7 +114,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="170">
   <si>
     <t>数据类型</t>
   </si>
@@ -590,6 +590,56 @@
     <t>专业代码，专业名称，进修年限，职业面向，培养目标，专业能力要求，专业课程与实训实习，职业证书类型，持续教育专业方向</t>
   </si>
   <si>
+    <t>课程资源</t>
+  </si>
+  <si>
+    <t>教材</t>
+  </si>
+  <si>
+    <t>面向课程教学、专业教学、职业教育或培训场景使用的教材、参考教材、讲义、实训教材、任务式教材、新形态教材等文档。通常具有书名、编者/主编、出版社、内容
+                             提要、目录、章节/项目/任务、学习目标、知识点、案例、训练题、实训任务、配套资源等结构。</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 教材知识库建设、课程资源检索、AI 助教问答、备课辅助、课程知识点抽取、教学设计辅助、职业能力与课程内容关联分析、Evidence Graph 上下文检索。</t>
+  </si>
+  <si>
+    <t>标题、封面或首页出现“教材”“职业教育教材”“改革创新教材”“新形态教材”“实训教材”“课程教材”“参考教材”等关键词。</t>
+  </si>
+  <si>
+    <t>正文出现“本书”“内容提要”“目录”“项目”“任务”“学习目标”“知识目标”“能力目标”“素质目标”“课后训练”“实训”“案例”“拓展资    思考、职业视窗、课后训练”等
+源”“扫码资源”等教材结构或教学栏目。出现出版社、编者/主编、出版地、ISBN、版次、印次、CIP、版权页等出版型文档信息。</t>
+  </si>
+  <si>
+    <t>从适用专业、课程归属、正文专业描述中抽取。</t>
+  </si>
+  <si>
+    <t>从“中职”“高职”“职业本科”“职业院校”“本科”等词汇抽取；仅出现“职业院校”时可标为泛化层次并待复核。</t>
+  </si>
+  <si>
+    <t>出版地、适用标准、政策依据、出版社归属等共同判断。</t>
+  </si>
+  <si>
+    <t>教材类默认按出版年份、版次、引用标准有效性判断；无法识别出版年份时标记为“需复核”。</t>
+  </si>
+  <si>
+    <t>文件来源、出版社、公开来源、内部上传来源共同判断。</t>
+  </si>
+  <si>
+    <t>出版社、主编、ISBN/CIP、版权页、官方资源页、来源链路越完整得分越高；仅文件名或未知来源得分降低。权重25%</t>
+  </si>
+  <si>
+    <t>3年内有效（依据：知识点、技能点的教学内容通常3年左右更新，符合行业发展节奏）。权重30%</t>
+  </si>
+  <si>
+    <t>应包含封面/书名、内容提要、目录、章节或项目正文、训练/实训/案例等主体内容；缺正文、缺目录、仅摘要则降分。权重35%</t>
+  </si>
+  <si>
+    <t>能识别章/项目/任务/小节、学习目标、知识点、案例、训练题、实训任务等层级</t>
+  </si>
+  <si>
+    <t>建议默认 L2。若确认是公开授权材料、公开样章或可开放传播内容，可降为 L1；若为校内未公开教材、内部讲义、含教师私有教案或版权受限全文，应保持 L2 或提升至 L3 并触发授权/使用范围复核。</t>
+  </si>
+  <si>
     <t>专业领域标签集：</t>
   </si>
   <si>
@@ -1053,7 +1103,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -1130,6 +1180,32 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1256,7 +1332,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1268,34 +1344,34 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1380,7 +1456,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1443,10 +1519,28 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" indent="2"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1768,7 +1862,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:R22"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.1627906976744" style="1" customWidth="1"/>
@@ -2364,84 +2458,327 @@
       </c>
     </row>
     <row r="13" ht="121.5" customHeight="1" spans="1:18">
-      <c r="A13" s="19"/>
-      <c r="B13" s="16" t="s">
+      <c r="A13" s="22"/>
+      <c r="B13" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="23" t="s">
         <v>130</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="E13" s="16" t="s">
+      <c r="E13" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="F13" s="16" t="s">
+      <c r="F13" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="16" t="s">
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="J13" s="16" t="s">
+      <c r="J13" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="K13" s="16" t="s">
+      <c r="K13" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="L13" s="16" t="s">
+      <c r="L13" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="M13" s="16" t="s">
+      <c r="M13" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="N13" s="16" t="s">
+      <c r="N13" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="O13" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="P13" s="17" t="s">
+      <c r="O13" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="P13" s="25" t="s">
         <v>99</v>
       </c>
       <c r="Q13" s="21" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="14" customHeight="1" spans="1:18">
-      <c r="G14" s="22"/>
-      <c r="H14" s="22"/>
-      <c r="I14" s="22"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="22"/>
-      <c r="L14" s="22"/>
-      <c r="M14" s="23"/>
-      <c r="N14" s="23"/>
-      <c r="O14" s="23"/>
-    </row>
-    <row r="15" ht="14.25" customHeight="1"/>
+    <row r="14" ht="268.3" spans="1:18">
+      <c r="A14" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="B14" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="C14" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="D14" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="E14" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="F14" s="27" t="s">
+        <v>146</v>
+      </c>
+      <c r="G14" s="28" t="s">
+        <v>147</v>
+      </c>
+      <c r="H14" s="28" t="s">
+        <v>148</v>
+      </c>
+      <c r="I14" s="28" t="s">
+        <v>149</v>
+      </c>
+      <c r="J14" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="K14" s="28" t="s">
+        <v>151</v>
+      </c>
+      <c r="L14" s="28" t="s">
+        <v>152</v>
+      </c>
+      <c r="M14" s="28" t="s">
+        <v>153</v>
+      </c>
+      <c r="N14" s="28" t="s">
+        <v>154</v>
+      </c>
+      <c r="O14" s="28" t="s">
+        <v>34</v>
+      </c>
+      <c r="P14" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q14" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="R14" s="27" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="15" ht="14.25" customHeight="1" spans="1:18">
+      <c r="A15" s="26"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
+      <c r="L15" s="27"/>
+      <c r="M15" s="27"/>
+      <c r="N15" s="27"/>
+      <c r="O15" s="27"/>
+      <c r="P15" s="26"/>
+      <c r="Q15" s="26"/>
+      <c r="R15" s="27"/>
+    </row>
     <row r="16" ht="14.25" customHeight="1" spans="1:18">
-      <c r="H16" s="3"/>
-    </row>
-    <row r="17" ht="14.25" customHeight="1" spans="8:8">
-      <c r="H17" s="3"/>
-    </row>
-    <row r="18" ht="14.25" customHeight="1" spans="8:8">
-      <c r="H18" s="3"/>
-    </row>
-    <row r="19" ht="14.25" customHeight="1" spans="8:8">
-      <c r="H19" s="3"/>
-    </row>
-    <row r="20" ht="14.25" customHeight="1" spans="8:8">
-      <c r="H20" s="3"/>
-    </row>
-    <row r="21" customHeight="1" spans="8:8">
-      <c r="H21" s="3"/>
-    </row>
-    <row r="22" customHeight="1" spans="8:8">
-      <c r="H22" s="3"/>
+      <c r="A16" s="26"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="27"/>
+      <c r="K16" s="27"/>
+      <c r="L16" s="27"/>
+      <c r="M16" s="27"/>
+      <c r="N16" s="27"/>
+      <c r="O16" s="27"/>
+      <c r="P16" s="26"/>
+      <c r="Q16" s="26"/>
+      <c r="R16" s="27"/>
+    </row>
+    <row r="17" ht="14.25" customHeight="1" spans="1:18">
+      <c r="A17" s="26"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="29"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="27"/>
+      <c r="K17" s="27"/>
+      <c r="L17" s="27"/>
+      <c r="M17" s="27"/>
+      <c r="N17" s="27"/>
+      <c r="O17" s="27"/>
+      <c r="P17" s="26"/>
+      <c r="Q17" s="26"/>
+      <c r="R17" s="27"/>
+    </row>
+    <row r="18" ht="14.25" customHeight="1" spans="1:18">
+      <c r="A18" s="26"/>
+      <c r="B18" s="27"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="29"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="27"/>
+      <c r="K18" s="27"/>
+      <c r="L18" s="27"/>
+      <c r="M18" s="27"/>
+      <c r="N18" s="27"/>
+      <c r="O18" s="27"/>
+      <c r="P18" s="26"/>
+      <c r="Q18" s="26"/>
+      <c r="R18" s="27"/>
+    </row>
+    <row r="19" ht="14.25" customHeight="1" spans="1:18">
+      <c r="A19" s="26"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
+      <c r="L19" s="27"/>
+      <c r="M19" s="27"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="27"/>
+      <c r="P19" s="26"/>
+      <c r="Q19" s="26"/>
+      <c r="R19" s="27"/>
+    </row>
+    <row r="20" ht="14.25" customHeight="1" spans="1:18">
+      <c r="A20" s="26"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="27"/>
+      <c r="K20" s="27"/>
+      <c r="L20" s="27"/>
+      <c r="M20" s="27"/>
+      <c r="N20" s="27"/>
+      <c r="O20" s="27"/>
+      <c r="P20" s="26"/>
+      <c r="Q20" s="26"/>
+      <c r="R20" s="27"/>
+    </row>
+    <row r="21" customHeight="1" spans="1:18">
+      <c r="A21" s="26"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="29"/>
+      <c r="I21" s="27"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
+      <c r="L21" s="27"/>
+      <c r="M21" s="27"/>
+      <c r="N21" s="27"/>
+      <c r="O21" s="27"/>
+      <c r="P21" s="26"/>
+      <c r="Q21" s="26"/>
+      <c r="R21" s="27"/>
+    </row>
+    <row r="22" customHeight="1" spans="1:18">
+      <c r="A22" s="26"/>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="27"/>
+      <c r="K22" s="27"/>
+      <c r="L22" s="27"/>
+      <c r="M22" s="27"/>
+      <c r="N22" s="27"/>
+      <c r="O22" s="27"/>
+      <c r="P22" s="26"/>
+      <c r="Q22" s="26"/>
+      <c r="R22" s="27"/>
+    </row>
+    <row r="23" customHeight="1" spans="1:18">
+      <c r="A23" s="26"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="27"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
+      <c r="L23" s="27"/>
+      <c r="M23" s="27"/>
+      <c r="N23" s="27"/>
+      <c r="O23" s="27"/>
+      <c r="P23" s="26"/>
+      <c r="Q23" s="26"/>
+      <c r="R23" s="27"/>
+    </row>
+    <row r="24" customHeight="1" spans="1:18">
+      <c r="A24" s="26"/>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="27"/>
+      <c r="J24" s="27"/>
+      <c r="K24" s="27"/>
+      <c r="L24" s="27"/>
+      <c r="M24" s="27"/>
+      <c r="N24" s="27"/>
+      <c r="O24" s="27"/>
+      <c r="P24" s="26"/>
+      <c r="Q24" s="26"/>
+      <c r="R24" s="27"/>
+    </row>
+    <row r="25" customHeight="1" spans="1:18">
+      <c r="A25" s="26"/>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="27"/>
+      <c r="I25" s="27"/>
+      <c r="J25" s="27"/>
+      <c r="K25" s="27"/>
+      <c r="L25" s="27"/>
+      <c r="M25" s="27"/>
+      <c r="N25" s="27"/>
+      <c r="O25" s="27"/>
+      <c r="P25" s="26"/>
+      <c r="Q25" s="26"/>
+      <c r="R25" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -2449,10 +2786,10 @@
     <mergeCell ref="G1:K1"/>
     <mergeCell ref="L1:O1"/>
     <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="L14:O14"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="A9:A13"/>
+    <mergeCell ref="A14:A25"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="G9:G13"/>
@@ -2480,42 +2817,42 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>144</v>
+        <v>160</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>145</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>146</v>
+        <v>162</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>27</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>148</v>
+        <v>164</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2"/>
       <c r="B3" s="3" t="s">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -2524,7 +2861,7 @@
     <row r="4" spans="1:5">
       <c r="A4" s="2"/>
       <c r="B4" s="3" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -2533,7 +2870,7 @@
     <row r="5" spans="1:5">
       <c r="A5" s="2"/>
       <c r="B5" s="3" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -2542,7 +2879,7 @@
     <row r="6" spans="1:5">
       <c r="A6" s="2"/>
       <c r="B6" s="3" t="s">
-        <v>153</v>
+        <v>169</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>

</xml_diff>

<commit_message>
feat(crawler): filter web shell noise before ingestion
</commit_message>
<xml_diff>
--- a/docs/ai-governance/20260605数据清单.xlsx
+++ b/docs/ai-governance/20260605数据清单.xlsx
@@ -114,7 +114,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="187">
   <si>
     <t>数据类型</t>
   </si>
@@ -640,6 +640,57 @@
     <t>建议默认 L2。若确认是公开授权材料、公开样章或可开放传播内容，可降为 L1；若为校内未公开教材、内部讲义、含教师私有教案或版权受限全文，应保持 L2 或提升至 L3 并触发授权/使用范围复核。</t>
   </si>
   <si>
+    <t>课程标准</t>
+  </si>
+  <si>
+    <t>各专业、各课程的课程标准、课程简介</t>
+  </si>
+  <si>
+    <t>AI助教、教材及课程生成、RAG知识库</t>
+  </si>
+  <si>
+    <t>课程标准；课程简介；精品课程建设；课程开发</t>
+  </si>
+  <si>
+    <t>课程定位；课程目标；课程模块结构；课程资源；教学方案；教学评价</t>
+  </si>
+  <si>
+    <t>3年内有效（依据：知识点、技能点的教学内容通常3年左右更新，符合行业发展节奏）</t>
+  </si>
+  <si>
+    <t>内容匹配度25%：直接对应专业教学标准中的课程名称、课程内容介绍，可直接复用</t>
+  </si>
+  <si>
+    <t>规范完整度25%：符合课程标准一般格式规范，结构完整</t>
+  </si>
+  <si>
+    <t>时效性25%：3年内的最新实训指导书，符合当前电商行业技术发展和实训教学改革的最新要求</t>
+  </si>
+  <si>
+    <t>落地性25%：可直接用于专业教学指导、实训项目设计、课程资源开发</t>
+  </si>
+  <si>
+    <t>案例</t>
+  </si>
+  <si>
+    <t>教学案例</t>
+  </si>
+  <si>
+    <t>教学案例；课堂案例；企业案例；项目案例</t>
+  </si>
+  <si>
+    <t>案例背景、案例分析、任务实施、成果展示、总结反思、评价方式</t>
+  </si>
+  <si>
+    <t>内容匹配度35%：直接对应电商专业课堂教学、实训教学的核心需求，可直接复用</t>
+  </si>
+  <si>
+    <t>时效性35%：3年内的最新教学案例，符合当前电商行业发展和教学改革的最新要求</t>
+  </si>
+  <si>
+    <t>落地性30%：可直接用于课堂教学、实训项目设计、课程资源开发、教师教学能力提升</t>
+  </si>
+  <si>
     <t>专业领域标签集：</t>
   </si>
   <si>
@@ -689,7 +740,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="32">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -740,6 +791,12 @@
       <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -1326,137 +1383,137 @@
     <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1530,12 +1587,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2505,280 +2568,328 @@
       </c>
     </row>
     <row r="14" ht="268.3" spans="1:18">
-      <c r="A14" s="26" t="s">
+      <c r="A14" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="26" t="s">
         <v>142</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="D14" s="27" t="s">
+      <c r="D14" s="26" t="s">
         <v>144</v>
       </c>
-      <c r="E14" s="27" t="s">
+      <c r="E14" s="26" t="s">
         <v>145</v>
       </c>
-      <c r="F14" s="27" t="s">
+      <c r="F14" s="26" t="s">
         <v>146</v>
       </c>
-      <c r="G14" s="28" t="s">
+      <c r="G14" s="27" t="s">
         <v>147</v>
       </c>
-      <c r="H14" s="28" t="s">
+      <c r="H14" s="27" t="s">
         <v>148</v>
       </c>
-      <c r="I14" s="28" t="s">
+      <c r="I14" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="J14" s="28" t="s">
+      <c r="J14" s="27" t="s">
         <v>150</v>
       </c>
-      <c r="K14" s="28" t="s">
+      <c r="K14" s="27" t="s">
         <v>151</v>
       </c>
-      <c r="L14" s="28" t="s">
+      <c r="L14" s="27" t="s">
         <v>152</v>
       </c>
-      <c r="M14" s="28" t="s">
+      <c r="M14" s="27" t="s">
         <v>153</v>
       </c>
-      <c r="N14" s="28" t="s">
+      <c r="N14" s="27" t="s">
         <v>154</v>
       </c>
-      <c r="O14" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="P14" s="26" t="s">
+      <c r="O14" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="P14" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="Q14" s="26" t="s">
+      <c r="Q14" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="R14" s="27" t="s">
+      <c r="R14" s="26" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="15" ht="14.25" customHeight="1" spans="1:18">
-      <c r="A15" s="26"/>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="27"/>
-      <c r="K15" s="27"/>
-      <c r="L15" s="27"/>
-      <c r="M15" s="27"/>
-      <c r="N15" s="27"/>
-      <c r="O15" s="27"/>
-      <c r="P15" s="26"/>
-      <c r="Q15" s="26"/>
-      <c r="R15" s="27"/>
-    </row>
-    <row r="16" ht="14.25" customHeight="1" spans="1:18">
-      <c r="A16" s="26"/>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="29"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="27"/>
-      <c r="K16" s="27"/>
-      <c r="L16" s="27"/>
-      <c r="M16" s="27"/>
-      <c r="N16" s="27"/>
-      <c r="O16" s="27"/>
-      <c r="P16" s="26"/>
-      <c r="Q16" s="26"/>
-      <c r="R16" s="27"/>
+    <row r="15" ht="84.85" spans="1:18">
+      <c r="A15" s="18"/>
+      <c r="B15" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C15" s="28" t="s">
+        <v>158</v>
+      </c>
+      <c r="D15" s="29" t="s">
+        <v>159</v>
+      </c>
+      <c r="E15" s="29" t="s">
+        <v>160</v>
+      </c>
+      <c r="F15" s="29" t="s">
+        <v>161</v>
+      </c>
+      <c r="G15" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="H15" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="I15" s="26"/>
+      <c r="J15" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="K15" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="L15" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="M15" s="29" t="s">
+        <v>165</v>
+      </c>
+      <c r="N15" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="O15" s="26"/>
+      <c r="P15" s="18"/>
+      <c r="Q15" s="18"/>
+      <c r="R15" s="26"/>
+    </row>
+    <row r="16" ht="84.85" spans="1:18">
+      <c r="A16" s="18"/>
+      <c r="B16" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="C16" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="D16" s="29" t="s">
+        <v>159</v>
+      </c>
+      <c r="E16" s="29" t="s">
+        <v>169</v>
+      </c>
+      <c r="F16" s="29" t="s">
+        <v>170</v>
+      </c>
+      <c r="G16" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="H16" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="I16" s="26"/>
+      <c r="J16" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="K16" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="L16" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="M16" s="29" t="s">
+        <v>172</v>
+      </c>
+      <c r="N16" s="30" t="s">
+        <v>173</v>
+      </c>
+      <c r="O16" s="26"/>
+      <c r="P16" s="18"/>
+      <c r="Q16" s="18"/>
+      <c r="R16" s="26"/>
     </row>
     <row r="17" ht="14.25" customHeight="1" spans="1:18">
-      <c r="A17" s="26"/>
-      <c r="B17" s="27"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="29"/>
-      <c r="I17" s="27"/>
-      <c r="J17" s="27"/>
-      <c r="K17" s="27"/>
-      <c r="L17" s="27"/>
-      <c r="M17" s="27"/>
-      <c r="N17" s="27"/>
-      <c r="O17" s="27"/>
-      <c r="P17" s="26"/>
-      <c r="Q17" s="26"/>
-      <c r="R17" s="27"/>
+      <c r="A17" s="18"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="31"/>
+      <c r="I17" s="26"/>
+      <c r="J17" s="26"/>
+      <c r="K17" s="26"/>
+      <c r="L17" s="26"/>
+      <c r="M17" s="26"/>
+      <c r="N17" s="26"/>
+      <c r="O17" s="26"/>
+      <c r="P17" s="18"/>
+      <c r="Q17" s="18"/>
+      <c r="R17" s="26"/>
     </row>
     <row r="18" ht="14.25" customHeight="1" spans="1:18">
-      <c r="A18" s="26"/>
-      <c r="B18" s="27"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="27"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="29"/>
-      <c r="I18" s="27"/>
-      <c r="J18" s="27"/>
-      <c r="K18" s="27"/>
-      <c r="L18" s="27"/>
-      <c r="M18" s="27"/>
-      <c r="N18" s="27"/>
-      <c r="O18" s="27"/>
-      <c r="P18" s="26"/>
-      <c r="Q18" s="26"/>
-      <c r="R18" s="27"/>
+      <c r="A18" s="18"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="26"/>
+      <c r="J18" s="26"/>
+      <c r="K18" s="26"/>
+      <c r="L18" s="26"/>
+      <c r="M18" s="26"/>
+      <c r="N18" s="26"/>
+      <c r="O18" s="26"/>
+      <c r="P18" s="18"/>
+      <c r="Q18" s="18"/>
+      <c r="R18" s="26"/>
     </row>
     <row r="19" ht="14.25" customHeight="1" spans="1:18">
-      <c r="A19" s="26"/>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="29"/>
-      <c r="I19" s="27"/>
-      <c r="J19" s="27"/>
-      <c r="K19" s="27"/>
-      <c r="L19" s="27"/>
-      <c r="M19" s="27"/>
-      <c r="N19" s="27"/>
-      <c r="O19" s="27"/>
-      <c r="P19" s="26"/>
-      <c r="Q19" s="26"/>
-      <c r="R19" s="27"/>
+      <c r="A19" s="18"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="31"/>
+      <c r="I19" s="26"/>
+      <c r="J19" s="26"/>
+      <c r="K19" s="26"/>
+      <c r="L19" s="26"/>
+      <c r="M19" s="26"/>
+      <c r="N19" s="26"/>
+      <c r="O19" s="26"/>
+      <c r="P19" s="18"/>
+      <c r="Q19" s="18"/>
+      <c r="R19" s="26"/>
     </row>
     <row r="20" ht="14.25" customHeight="1" spans="1:18">
-      <c r="A20" s="26"/>
-      <c r="B20" s="27"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="29"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="27"/>
-      <c r="K20" s="27"/>
-      <c r="L20" s="27"/>
-      <c r="M20" s="27"/>
-      <c r="N20" s="27"/>
-      <c r="O20" s="27"/>
-      <c r="P20" s="26"/>
-      <c r="Q20" s="26"/>
-      <c r="R20" s="27"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="26"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="31"/>
+      <c r="I20" s="26"/>
+      <c r="J20" s="26"/>
+      <c r="K20" s="26"/>
+      <c r="L20" s="26"/>
+      <c r="M20" s="26"/>
+      <c r="N20" s="26"/>
+      <c r="O20" s="26"/>
+      <c r="P20" s="18"/>
+      <c r="Q20" s="18"/>
+      <c r="R20" s="26"/>
     </row>
     <row r="21" customHeight="1" spans="1:18">
-      <c r="A21" s="26"/>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="29"/>
-      <c r="I21" s="27"/>
-      <c r="J21" s="27"/>
-      <c r="K21" s="27"/>
-      <c r="L21" s="27"/>
-      <c r="M21" s="27"/>
-      <c r="N21" s="27"/>
-      <c r="O21" s="27"/>
-      <c r="P21" s="26"/>
-      <c r="Q21" s="26"/>
-      <c r="R21" s="27"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="26"/>
+      <c r="K21" s="26"/>
+      <c r="L21" s="26"/>
+      <c r="M21" s="26"/>
+      <c r="N21" s="26"/>
+      <c r="O21" s="26"/>
+      <c r="P21" s="18"/>
+      <c r="Q21" s="18"/>
+      <c r="R21" s="26"/>
     </row>
     <row r="22" customHeight="1" spans="1:18">
-      <c r="A22" s="26"/>
-      <c r="B22" s="27"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="29"/>
-      <c r="I22" s="27"/>
-      <c r="J22" s="27"/>
-      <c r="K22" s="27"/>
-      <c r="L22" s="27"/>
-      <c r="M22" s="27"/>
-      <c r="N22" s="27"/>
-      <c r="O22" s="27"/>
-      <c r="P22" s="26"/>
-      <c r="Q22" s="26"/>
-      <c r="R22" s="27"/>
+      <c r="A22" s="18"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="31"/>
+      <c r="I22" s="26"/>
+      <c r="J22" s="26"/>
+      <c r="K22" s="26"/>
+      <c r="L22" s="26"/>
+      <c r="M22" s="26"/>
+      <c r="N22" s="26"/>
+      <c r="O22" s="26"/>
+      <c r="P22" s="18"/>
+      <c r="Q22" s="18"/>
+      <c r="R22" s="26"/>
     </row>
     <row r="23" customHeight="1" spans="1:18">
-      <c r="A23" s="26"/>
-      <c r="B23" s="27"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="27"/>
-      <c r="I23" s="27"/>
-      <c r="J23" s="27"/>
-      <c r="K23" s="27"/>
-      <c r="L23" s="27"/>
-      <c r="M23" s="27"/>
-      <c r="N23" s="27"/>
-      <c r="O23" s="27"/>
-      <c r="P23" s="26"/>
-      <c r="Q23" s="26"/>
-      <c r="R23" s="27"/>
+      <c r="A23" s="18"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
+      <c r="J23" s="26"/>
+      <c r="K23" s="26"/>
+      <c r="L23" s="26"/>
+      <c r="M23" s="26"/>
+      <c r="N23" s="26"/>
+      <c r="O23" s="26"/>
+      <c r="P23" s="18"/>
+      <c r="Q23" s="18"/>
+      <c r="R23" s="26"/>
     </row>
     <row r="24" customHeight="1" spans="1:18">
-      <c r="A24" s="26"/>
-      <c r="B24" s="27"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="27"/>
-      <c r="I24" s="27"/>
-      <c r="J24" s="27"/>
-      <c r="K24" s="27"/>
-      <c r="L24" s="27"/>
-      <c r="M24" s="27"/>
-      <c r="N24" s="27"/>
-      <c r="O24" s="27"/>
-      <c r="P24" s="26"/>
-      <c r="Q24" s="26"/>
-      <c r="R24" s="27"/>
+      <c r="A24" s="18"/>
+      <c r="B24" s="26"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="26"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="26"/>
+      <c r="K24" s="26"/>
+      <c r="L24" s="26"/>
+      <c r="M24" s="26"/>
+      <c r="N24" s="26"/>
+      <c r="O24" s="26"/>
+      <c r="P24" s="18"/>
+      <c r="Q24" s="18"/>
+      <c r="R24" s="26"/>
     </row>
     <row r="25" customHeight="1" spans="1:18">
-      <c r="A25" s="26"/>
-      <c r="B25" s="27"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="27"/>
-      <c r="F25" s="27"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="27"/>
-      <c r="I25" s="27"/>
-      <c r="J25" s="27"/>
-      <c r="K25" s="27"/>
-      <c r="L25" s="27"/>
-      <c r="M25" s="27"/>
-      <c r="N25" s="27"/>
-      <c r="O25" s="27"/>
-      <c r="P25" s="26"/>
-      <c r="Q25" s="26"/>
-      <c r="R25" s="27"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="26"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="26"/>
+      <c r="G25" s="26"/>
+      <c r="H25" s="26"/>
+      <c r="I25" s="26"/>
+      <c r="J25" s="26"/>
+      <c r="K25" s="26"/>
+      <c r="L25" s="26"/>
+      <c r="M25" s="26"/>
+      <c r="N25" s="26"/>
+      <c r="O25" s="26"/>
+      <c r="P25" s="18"/>
+      <c r="Q25" s="18"/>
+      <c r="R25" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -2817,42 +2928,42 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>157</v>
+        <v>174</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>158</v>
+        <v>175</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>159</v>
+        <v>176</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>27</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>163</v>
+        <v>180</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>164</v>
+        <v>181</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2"/>
       <c r="B3" s="3" t="s">
-        <v>166</v>
+        <v>183</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -2861,7 +2972,7 @@
     <row r="4" spans="1:5">
       <c r="A4" s="2"/>
       <c r="B4" s="3" t="s">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -2870,7 +2981,7 @@
     <row r="5" spans="1:5">
       <c r="A5" s="2"/>
       <c r="B5" s="3" t="s">
-        <v>168</v>
+        <v>185</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -2879,7 +2990,7 @@
     <row r="6" spans="1:5">
       <c r="A6" s="2"/>
       <c r="B6" s="3" t="s">
-        <v>169</v>
+        <v>186</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>

</xml_diff>